<commit_message>
docs: add EMM-03-A2 state vector implementation plan & sync core files
</commit_message>
<xml_diff>
--- a/emma_jira_tracker.xlsx
+++ b/emma_jira_tracker.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="139">
   <si>
     <t>Ticket ID</t>
   </si>
@@ -425,13 +425,19 @@
   </si>
   <si>
     <t xml:space="preserve">   DONE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   DONE </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> DONE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -479,8 +485,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -534,6 +547,30 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -570,13 +607,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -611,10 +652,26 @@
     <xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="2" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="2" xfId="7" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="8">
+    <cellStyle name="40% - Accent4" xfId="5" builtinId="43"/>
+    <cellStyle name="40% - Accent5" xfId="6" builtinId="47"/>
     <cellStyle name="60% - Accent1" xfId="2" builtinId="32"/>
     <cellStyle name="60% - Accent3" xfId="3" builtinId="40"/>
+    <cellStyle name="60% - Accent5" xfId="7" builtinId="48"/>
+    <cellStyle name="60% - Accent6" xfId="4" builtinId="52"/>
     <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -1098,6 +1155,9 @@
       <c r="M4" s="3" t="s">
         <v>37</v>
       </c>
+      <c r="N4" s="12" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="5" spans="1:14" ht="15" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
@@ -1139,6 +1199,9 @@
       <c r="M5" s="7" t="s">
         <v>43</v>
       </c>
+      <c r="N5" s="13" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="6" spans="1:14" ht="15" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
@@ -1180,6 +1243,9 @@
       <c r="M6" s="3" t="s">
         <v>50</v>
       </c>
+      <c r="N6" s="14" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="7" spans="1:14" ht="15" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
@@ -1220,6 +1286,9 @@
       </c>
       <c r="M7" s="7" t="s">
         <v>57</v>
+      </c>
+      <c r="N7" s="15" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="15" x14ac:dyDescent="0.3">

</xml_diff>